<commit_message>
polishing and logic fixing
</commit_message>
<xml_diff>
--- a/annual_health_checkup_automation/Hospital_Employee_Roster_Dummy.xlsx
+++ b/annual_health_checkup_automation/Hospital_Employee_Roster_Dummy.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikhi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikhi\Downloads\automation-and-tools-for-HR\annual_health_checkup_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC40117C-9CF9-4568-98FD-616C49E2C827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C675AF9D-4354-449B-8C70-7FF90358975D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="144">
   <si>
     <t>Employee ID</t>
   </si>
@@ -79,6 +79,9 @@
     <t>Employment Type</t>
   </si>
   <si>
+    <t>Last Working Day (LWD)</t>
+  </si>
+  <si>
     <t>Checkup Date</t>
   </si>
   <si>
@@ -482,6 +485,9 @@
   </si>
   <si>
     <t>Sanjay Shetty</t>
+  </si>
+  <si>
+    <t>Email ID</t>
   </si>
 </sst>
 </file>
@@ -543,13 +549,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -814,7 +821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -825,9 +832,10 @@
     <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -850,33 +858,39 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K1" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" s="3">
         <v>45488</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" s="3">
         <v>45778</v>
@@ -884,55 +898,63 @@
       <c r="I2" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J2" s="4">
+        <v>45813</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" s="3">
         <v>45358</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="H3" s="3">
+        <v>45779</v>
+      </c>
       <c r="I3" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J3" s="4">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4" s="3">
         <v>44006</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="3">
         <v>45695</v>
@@ -940,28 +962,31 @@
       <c r="I4" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J4" s="4">
+        <v>45272</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F5" s="3">
         <v>43523</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H5" s="3">
         <v>46119</v>
@@ -969,28 +994,31 @@
       <c r="I5" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J5" s="4">
+        <v>43787</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F6" s="3">
         <v>45008</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H6" s="3">
         <v>45813</v>
@@ -998,28 +1026,31 @@
       <c r="I6" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J6" s="4">
+        <v>45915</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F7" s="3">
         <v>44507</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H7" s="3">
         <v>45633</v>
@@ -1027,28 +1058,31 @@
       <c r="I7" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J7" s="4">
+        <v>44358</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F8" s="3">
         <v>43261</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H8" s="3">
         <v>46145</v>
@@ -1056,28 +1090,31 @@
       <c r="I8" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J8" s="4">
+        <v>43782</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F9" s="3">
         <v>43484</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H9" s="3">
         <v>46239</v>
@@ -1085,55 +1122,63 @@
       <c r="I9" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J9" s="4">
+        <v>43783</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F10" s="3">
         <v>45839</v>
       </c>
       <c r="G10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="3">
+        <v>46240</v>
+      </c>
+      <c r="I10" s="2">
+        <v>1</v>
+      </c>
+      <c r="J10" s="4">
+        <v>43784</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="F11" s="3">
         <v>43994</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H11" s="3">
         <v>45812</v>
@@ -1141,28 +1186,31 @@
       <c r="I11" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J11" s="4">
+        <v>43785</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F12" s="3">
         <v>45351</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H12" s="3">
         <v>45999</v>
@@ -1170,28 +1218,31 @@
       <c r="I12" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J12" s="4">
+        <v>43786</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F13" s="3">
         <v>43440</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H13" s="3">
         <v>46233</v>
@@ -1199,28 +1250,31 @@
       <c r="I13" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J13" s="4">
+        <v>43787</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F14" s="3">
         <v>43117</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H14" s="3">
         <v>45937</v>
@@ -1228,28 +1282,31 @@
       <c r="I14" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J14" s="4">
+        <v>43788</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F15" s="3">
         <v>45888</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H15" s="3">
         <v>45962</v>
@@ -1257,109 +1314,127 @@
       <c r="I15" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J15" s="4">
+        <v>43789</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F16" s="3">
         <v>44905</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H16" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="H16" s="3">
+        <v>45963</v>
+      </c>
       <c r="I16" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J16" s="4">
+        <v>43790</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F17" s="3">
         <v>44590</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H17" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="H17" s="3">
+        <v>45964</v>
+      </c>
       <c r="I17" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J17" s="4">
+        <v>43791</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F18" s="3">
         <v>45043</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H18" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="H18" s="3">
+        <v>45965</v>
+      </c>
       <c r="I18" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J18" s="4">
+        <v>43792</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F19" s="3">
         <v>43519</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H19" s="3">
         <v>46049</v>
@@ -1367,28 +1442,31 @@
       <c r="I19" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J19" s="4">
+        <v>43793</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F20" s="3">
         <v>45927</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H20" s="3">
         <v>45864</v>
@@ -1396,28 +1474,31 @@
       <c r="I20" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J20" s="4">
+        <v>43794</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F21" s="3">
         <v>44013</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H21" s="3">
         <v>46186</v>
@@ -1425,28 +1506,31 @@
       <c r="I21" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J21" s="4">
+        <v>43795</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F22" s="3">
         <v>46095</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H22" s="3">
         <v>45845</v>
@@ -1454,28 +1538,32 @@
       <c r="I22" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J22" s="4">
+        <f ca="1">IF(RAND()&lt;0.35,"",TODAY()-RANDBETWEEN(30,2800))</f>
+        <v>44544</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F23" s="3">
         <v>44594</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H23" s="3">
         <v>45791</v>
@@ -1483,28 +1571,32 @@
       <c r="I23" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J23" s="4">
+        <f t="shared" ref="J23:J46" ca="1" si="0">IF(RAND()&lt;0.35,"",TODAY()-RANDBETWEEN(30,2800))</f>
+        <v>45898</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F24" s="3">
         <v>45775</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H24" s="3">
         <v>45645</v>
@@ -1512,55 +1604,65 @@
       <c r="I24" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J24" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>45491</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F25" s="3">
         <v>45705</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H25" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="H25" s="3">
+        <v>45646</v>
+      </c>
       <c r="I25" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J25" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F26" s="3">
         <v>43213</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H26" s="3">
         <v>46035</v>
@@ -1568,28 +1670,32 @@
       <c r="I26" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J26" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F27" s="3">
         <v>43159</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H27" s="3">
         <v>45701</v>
@@ -1597,28 +1703,32 @@
       <c r="I27" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J27" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F28" s="3">
         <v>45153</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H28" s="3">
         <v>45892</v>
@@ -1626,28 +1736,32 @@
       <c r="I28" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J28" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>44822</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F29" s="3">
         <v>45814</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H29" s="3">
         <v>46072</v>
@@ -1655,28 +1769,32 @@
       <c r="I29" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J29" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F30" s="3">
         <v>43851</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H30" s="3">
         <v>45712</v>
@@ -1684,28 +1802,32 @@
       <c r="I30" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J30" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F31" s="3">
         <v>45895</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H31" s="3">
         <v>45667</v>
@@ -1713,28 +1835,32 @@
       <c r="I31" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J31" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F32" s="3">
         <v>45180</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H32" s="3">
         <v>45982</v>
@@ -1742,55 +1868,65 @@
       <c r="I32" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J32" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>45211</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F33" s="3">
         <v>44000</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H33" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="H33" s="3">
+        <v>45983</v>
+      </c>
       <c r="I33" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J33" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>43737</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F34" s="3">
         <v>44208</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H34" s="3">
         <v>45340</v>
@@ -1798,28 +1934,32 @@
       <c r="I34" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J34" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>45821</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F35" s="3">
         <v>43762</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H35" s="3">
         <v>44567</v>
@@ -1827,28 +1967,32 @@
       <c r="I35" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J35" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>46055</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F36" s="3">
         <v>44758</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H36" s="3">
         <v>45074</v>
@@ -1856,82 +2000,98 @@
       <c r="I36" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J36" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>45533</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F37" s="3">
         <v>45045</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H37" s="2"/>
+        <v>26</v>
+      </c>
+      <c r="H37" s="3">
+        <v>45075</v>
+      </c>
       <c r="I37" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J37" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F38" s="3">
         <v>45912</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H38" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="H38" s="3">
+        <v>45076</v>
+      </c>
       <c r="I38" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J38" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>45921</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F39" s="3">
         <v>43415</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H39" s="3">
         <v>43590</v>
@@ -1939,28 +2099,32 @@
       <c r="I39" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J39" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>44470</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F40" s="3">
         <v>44685</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H40" s="3">
         <v>45115</v>
@@ -1968,55 +2132,65 @@
       <c r="I40" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J40" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F41" s="3">
         <v>46021</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H41" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="H41" s="3">
+        <v>45116</v>
+      </c>
       <c r="I41" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J41" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>45846</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F42" s="3">
         <v>45740</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H42" s="3">
         <v>45910</v>
@@ -2024,28 +2198,32 @@
       <c r="I42" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J42" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F43" s="3">
         <v>43816</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H43" s="3">
         <v>45138</v>
@@ -2053,28 +2231,32 @@
       <c r="I43" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J43" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>45322</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F44" s="3">
         <v>46007</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H44" s="3">
         <v>46142</v>
@@ -2082,61 +2264,75 @@
       <c r="I44" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J44" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F45" s="3">
         <v>44690</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H45" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="H45" s="3">
+        <v>46143</v>
+      </c>
       <c r="I45" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J45" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>44719</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F46" s="3">
         <v>43912</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H46" s="3">
         <v>43950</v>
       </c>
       <c r="I46" s="2">
         <v>2</v>
+      </c>
+      <c r="J46" s="4" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>